<commit_message>
Minor bugfixes after last commit
</commit_message>
<xml_diff>
--- a/mapping.xlsx
+++ b/mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Desktop/Slovenija/Razširjeni kazalniki/streamlit_turisticne_regije_app_v4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA60F51-A01F-904E-AB30-997C14B4CD7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10F5527D-C95E-3D45-9459-3452C134A167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39500" yWindow="10000" windowWidth="39140" windowHeight="27100" xr2:uid="{E0B33F7B-3E2E-634E-A0CD-58CFEDBE8ACF}"/>
+    <workbookView xWindow="28340" yWindow="14880" windowWidth="39140" windowHeight="27100" xr2:uid="{E0B33F7B-3E2E-634E-A0CD-58CFEDBE8ACF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="182">
   <si>
     <t>Povprečna starost prebivalcev 2024</t>
   </si>
@@ -455,9 +455,6 @@
     <t>Nastanitvene kapacitete - stalna ležišča 2025</t>
   </si>
   <si>
-    <t>Število sob (ned.enot) v kapacitetah višje kakovosti -( 4* in 5*) 2025</t>
-  </si>
-  <si>
     <t>Povprečna letna zasedenost staln. Ležišč 2024</t>
   </si>
   <si>
@@ -579,6 +576,12 @@
   </si>
   <si>
     <t>Struktura nastanitvenih kapacitet - Sobe (nedeljive enote) - Kampi</t>
+  </si>
+  <si>
+    <t>Delež sob (ned.enot) v kapacitetah višje kakovosti - (4* in 5*) 2025</t>
+  </si>
+  <si>
+    <t>Število sob (ned.enot) v kapacitetah višje kakovosti - ( 4* in 5*) 2025</t>
   </si>
 </sst>
 </file>
@@ -637,8 +640,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{98C3FF97-646E-4345-ACD2-3DBDFB48C0DC}" name="Table3" displayName="Table3" ref="A1:D92" totalsRowShown="0">
-  <autoFilter ref="A1:D92" xr:uid="{98C3FF97-646E-4345-ACD2-3DBDFB48C0DC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{98C3FF97-646E-4345-ACD2-3DBDFB48C0DC}" name="Table3" displayName="Table3" ref="A1:D94" totalsRowShown="0">
+  <autoFilter ref="A1:D94" xr:uid="{98C3FF97-646E-4345-ACD2-3DBDFB48C0DC}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{E236CF5C-F272-D343-B6D2-232DEB83E64D}" name="Družbeni kazalniki"/>
     <tableColumn id="2" xr3:uid="{E061FFED-142A-4740-9F7F-5346A3756A7D}" name="Okoljski kazalniki"/>
@@ -966,7 +969,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E12D345-358A-1946-9FC4-9A3FAE83F964}">
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D91"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="71" bestFit="1" customWidth="1"/>
@@ -998,7 +1001,7 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>141</v>
+        <v>75</v>
       </c>
       <c r="D2" t="s">
         <v>34</v>
@@ -1009,10 +1012,10 @@
         <v>72</v>
       </c>
       <c r="B3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C3" t="s">
-        <v>142</v>
+        <v>76</v>
       </c>
       <c r="D3" t="s">
         <v>35</v>
@@ -1026,7 +1029,7 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>143</v>
+        <v>77</v>
       </c>
       <c r="D4" t="s">
         <v>37</v>
@@ -1037,10 +1040,10 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C5" t="s">
-        <v>177</v>
+        <v>78</v>
       </c>
       <c r="D5" t="s">
         <v>38</v>
@@ -1051,10 +1054,10 @@
         <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C6" t="s">
-        <v>178</v>
+        <v>79</v>
       </c>
       <c r="D6" t="s">
         <v>39</v>
@@ -1068,7 +1071,7 @@
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D7" t="s">
         <v>40</v>
@@ -1076,13 +1079,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B8" t="s">
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D8" t="s">
         <v>41</v>
@@ -1090,13 +1093,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D9" t="s">
         <v>42</v>
@@ -1104,13 +1107,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B10" t="s">
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="D10" t="s">
         <v>43</v>
@@ -1118,13 +1121,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C11" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D11" t="s">
         <v>44</v>
@@ -1132,13 +1135,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D12" t="s">
         <v>45</v>
@@ -1146,10 +1149,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D13" t="s">
         <v>46</v>
@@ -1157,10 +1160,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C14" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D14" t="s">
         <v>47</v>
@@ -1168,10 +1171,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C15" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="D15" t="s">
         <v>48</v>
@@ -1179,10 +1182,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C16" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D16" t="s">
         <v>49</v>
@@ -1190,10 +1193,10 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C17" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D17" t="s">
         <v>50</v>
@@ -1201,10 +1204,10 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C18" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s">
         <v>51</v>
@@ -1212,10 +1215,10 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C19" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D19" t="s">
         <v>52</v>
@@ -1223,13 +1226,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C20" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -1237,7 +1240,7 @@
         <v>2</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D21" t="s">
         <v>53</v>
@@ -1245,10 +1248,10 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C22" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D22" t="s">
         <v>54</v>
@@ -1259,10 +1262,10 @@
         <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D23" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -1270,7 +1273,7 @@
         <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D24" t="s">
         <v>55</v>
@@ -1281,7 +1284,7 @@
         <v>6</v>
       </c>
       <c r="C25" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D25" t="s">
         <v>56</v>
@@ -1292,7 +1295,7 @@
         <v>7</v>
       </c>
       <c r="C26" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D26" t="s">
         <v>57</v>
@@ -1300,13 +1303,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C27" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D27" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -1314,7 +1317,7 @@
         <v>8</v>
       </c>
       <c r="C28" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D28" t="s">
         <v>58</v>
@@ -1322,10 +1325,10 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C29" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D29" t="s">
         <v>59</v>
@@ -1336,7 +1339,7 @@
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D30" t="s">
         <v>60</v>
@@ -1344,10 +1347,10 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C31" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D31" t="s">
         <v>61</v>
@@ -1355,10 +1358,10 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C32" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="D32" t="s">
         <v>62</v>
@@ -1366,61 +1369,67 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>4</v>
+        <v>176</v>
       </c>
       <c r="C33" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D33" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C34" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D34" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" t="s">
+        <v>107</v>
+      </c>
+      <c r="D35" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C35" t="s">
-        <v>102</v>
-      </c>
-      <c r="D35" t="s">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>175</v>
+      </c>
+      <c r="C36" t="s">
+        <v>108</v>
+      </c>
+      <c r="D36" t="s">
         <v>167</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C36" t="s">
-        <v>103</v>
-      </c>
-      <c r="D36" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C37" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D37" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C38" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="D38" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C39" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D39" t="s">
         <v>63</v>
@@ -1428,7 +1437,7 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C40" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D40" t="s">
         <v>64</v>
@@ -1436,7 +1445,7 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C41" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D41" t="s">
         <v>65</v>
@@ -1444,7 +1453,7 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C42" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D42" t="s">
         <v>36</v>
@@ -1452,255 +1461,250 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C43" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D43" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C44" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C45" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C46" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C47" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C48" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="49" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C49" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="50" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C50" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
     <row r="51" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C51" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="52" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C52" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="53" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C53" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="54" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C54" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="55" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C55" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="56" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C56" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="57" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C57" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="58" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C58" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="59" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C59" t="s">
-        <v>126</v>
+        <v>178</v>
       </c>
     </row>
     <row r="60" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C60" t="s">
-        <v>127</v>
+        <v>179</v>
       </c>
     </row>
     <row r="61" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C61" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="62" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C62" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="63" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C63" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="64" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C64" t="s">
-        <v>179</v>
+        <v>134</v>
       </c>
     </row>
     <row r="65" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C65" t="s">
-        <v>180</v>
+        <v>135</v>
       </c>
     </row>
     <row r="66" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C66" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="67" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C67" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="68" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C68" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="69" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C69" t="s">
-        <v>134</v>
+        <v>181</v>
       </c>
     </row>
     <row r="70" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C70" t="s">
-        <v>135</v>
+        <v>180</v>
       </c>
     </row>
     <row r="71" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C71" t="s">
-        <v>136</v>
+        <v>17</v>
       </c>
     </row>
     <row r="72" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C72" t="s">
-        <v>137</v>
+        <v>18</v>
       </c>
     </row>
     <row r="73" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C73" t="s">
-        <v>138</v>
+        <v>19</v>
       </c>
     </row>
     <row r="74" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C74" t="s">
-        <v>139</v>
+        <v>20</v>
       </c>
     </row>
     <row r="75" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C75" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="76" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C76" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="77" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C77" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="78" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C78" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="79" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C79" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="80" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C80" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="81" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C81" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="82" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C82" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="83" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C83" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="84" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C84" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="85" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C85" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="86" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C86" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="87" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C87" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="88" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C88" t="s">
-        <v>30</v>
+        <v>139</v>
       </c>
     </row>
     <row r="89" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C89" t="s">
-        <v>31</v>
+        <v>140</v>
       </c>
     </row>
     <row r="90" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C90" t="s">
-        <v>32</v>
+        <v>141</v>
       </c>
     </row>
     <row r="91" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C91" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="92" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C92" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>